<commit_message>
compare to data from DosSantos2020
</commit_message>
<xml_diff>
--- a/__EvoM1_TraitTable/brain_cortex_neurons_other_microglia.xlsx
+++ b/__EvoM1_TraitTable/brain_cortex_neurons_other_microglia.xlsx
@@ -3165,9 +3165,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D00FEA9A-1709-4A92-8BB6-371E918A3F55}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F45D03D-6EDB-4C91-97F9-AD927E3A04DF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{588CB5B3-92E4-4771-AAE9-5B445A3D75C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CAA1704-3F82-4838-A007-7DFB342E6CEE}"/>
 </file>
</xml_diff>